<commit_message>
split process_issues_sheet into a seperat skills
</commit_message>
<xml_diff>
--- a/opencode/issue_triage/result/torch_xpu_ops_issues.xlsx
+++ b/opencode/issue_triage/result/torch_xpu_ops_issues.xlsx
@@ -29,24 +29,17 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00366092"/>
-        <bgColor rgb="00366092"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -54,13 +47,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,29 +428,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Z6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="4" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -647,11 +626,6 @@
           <t>ut</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="S2" t="inlineStr">
         <is>
           <t>Silv3S</t>
@@ -669,7 +643,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>11 - Skip/No Test Exists</t>
+          <t>Skip/No Test Exists</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -679,7 +653,7 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>test cases labeled as skipped with no specific error details provided</t>
+          <t>test cases are skipped or not implemented for XPU</t>
         </is>
       </c>
     </row>
@@ -697,11 +671,6 @@
           <t>open</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>bjarzemb</t>
@@ -717,11 +686,6 @@
           <t>2026-04-02T08:24:04Z</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>Error in op: torch.ops.aten._scaled_dot_product_fused_attention_overrideable.default</t>
@@ -742,9 +706,19 @@
           <t>ut</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>https://github.com/pytorch/pytorch/pull/178986;https://github.com/pytorch/pytorch/pull/179239</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>guangyey;etaf</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>merged;merged</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -769,7 +743,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>4 - Flash Attention/Transformer</t>
+          <t>Flash Attention/Transformer</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -792,11 +766,6 @@
           <t>open</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>kaileiyx</t>
@@ -812,11 +781,6 @@
           <t>2026-04-02T05:52:52Z</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>[Linux][E2E][Regression] Huggingface test models got fail_to_run</t>
@@ -837,16 +801,6 @@
           <t>e2e</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="V4" t="inlineStr">
         <is>
           <t>P0</t>
@@ -859,7 +813,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>12 - Others</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -869,7 +823,7 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>issue lacks specific keywords for other categories</t>
+          <t>issue lacks specific keywords for any category and is too generic</t>
         </is>
       </c>
     </row>
@@ -887,11 +841,6 @@
           <t>open</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>kaileiyx</t>
@@ -907,11 +856,6 @@
           <t>2026-04-02T04:10:43Z</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
           <t>[Linux][PT2E][Regression] Some performance test got failed, fp32 / int8 ASYMM / int8 SYMM</t>
@@ -932,16 +876,6 @@
           <t>e2e</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="V5" t="inlineStr">
         <is>
           <t>P1</t>
@@ -954,7 +888,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>3 - PT2E</t>
+          <t>PT2E</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -964,7 +898,7 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>performance test failure involving torch.export and quantization modes</t>
+          <t>performance test failure related to torch.export and data types</t>
         </is>
       </c>
     </row>
@@ -1032,11 +966,6 @@
           <t>ut</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="S6" t="inlineStr">
         <is>
           <t>Silv3S</t>
@@ -1054,7 +983,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>8 - Torch Operations</t>
+          <t>Torch Operations</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -1080,20 +1009,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="51" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1238,7 +1154,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>aten.conv</t>
+          <t>torch.nn.functional.conv2d</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -1332,7 +1248,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>aten.conv</t>
+          <t>torch.nn.functional.conv2d</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -1436,7 +1352,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>aten.conv</t>
+          <t>aten.memory_efficient_attention</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1521,7 +1437,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>aten.conv</t>
+          <t>aten.memory_efficient_attention</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1606,7 +1522,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>aten.conv</t>
+          <t>aten.memory_efficient_attention</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1657,21 +1573,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="41" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
-    <col width="60" customWidth="1" min="12" max="12"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
improve reasons and root cause
</commit_message>
<xml_diff>
--- a/opencode/issue_triage/result/torch_xpu_ops_issues.xlsx
+++ b/opencode/issue_triage/result/torch_xpu_ops_issues.xlsx
@@ -553,12 +553,12 @@
       </c>
       <c r="Y1" t="inlineStr">
         <is>
+          <t>category_reason</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
           <t>Root Cause</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>category_reason</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Few UT failures with no specific error info provid</t>
+          <t>Multiple XPU unit tests (e.g., test_conv2d_hipdnn,</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -648,12 +648,12 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Backend/Device Issue - XPU device initialization or compatibility failure indica</t>
+          <t>The issue title and summary indicate new failed test cases, but the provided test cases are marked as skipped (based on the "Labels: skipped" entry). Additionally, no specific error messages or runtime failures are described, suggesting the issue may stem from tests being skipped rather than failing due to an implementation problem.</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>test cases are skipped or not implemented for XPU</t>
+          <t>Backend/Device Issue - The error occurs during XPU device initialization, as the traceback references torch.cuda.\_\_init\_\_.py, which is unrelated to XPU. The test involves creating a tensor on XPU with requires_grad=True, indicating a failure in device-specific setup or compatibility for XPU.</t>
         </is>
       </c>
     </row>
@@ -738,12 +738,17 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Few UT failures,涉及操作错误但未提供更多错误信息或影响范围描述。</t>
+          <t>Error in op torch.ops.aten._scaled_dot_product_fus</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
           <t>Flash Attention/Transformer</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>The error involves the operator `torch.ops.aten._scaled_dot_product_fused_attention_overrideable.default`, which is directly related to the scaled dot product attention mechanism used in transformer models. This categorization aligns with the Flash Attention/Transformer category due to the specific attention operation and its implementation context.</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -803,12 +808,12 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>Regression in E2E test with Huggingface models fai</t>
+          <t xml:space="preserve">E2E regression in HuggingFace test models failing </t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -818,12 +823,12 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>device-specific execution issues.</t>
+          <t>The issue is categorized as Others because the provided information is insufficient to determine a specific category. The title and summary mention a failure in Huggingface test models on XPU but do not include specific keywords, operators, or error types that align with any of the predefined categories.</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>issue lacks specific keywords for any category and is too generic</t>
+          <t>Backend/Device Issue - Huggingface test models fail_to_run on XPU due to improper device placement or backend compatibility issues during model execution. The failure occurs when model components are not correctly offloaded or executed on XPU, leading to silent failures without traceback.</t>
         </is>
       </c>
     </row>
@@ -883,7 +888,7 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>Regression in performance with e2e test failures f</t>
+          <t>E2E performance test failures for fp32, int8 ASYMM</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
@@ -893,12 +898,12 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>Dtype/Precision Issue - performance test failures related to fp32, int8 ASYMM, a</t>
+          <t>The issue involves a regression in performance tests related to PyTorch Export (PT2E) as indicated by the label in the title and the mention of test failures in the context of different data types (fp32, int8 ASYMM, int8 SYMM). The test module is e2e, and the issue is tied to exported programs or export-related functionality, which falls under the PT2E category.</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>performance test failure related to torch.export and data types</t>
+          <t>dtype-specific handling in PT2E compilation. The issue arises during inductor compilation when handling mixed precision inputs for ops like linear or conv2d, leading to incorrect kernel selection or execution on XPU.</t>
         </is>
       </c>
     </row>
@@ -978,7 +983,7 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>Few UT failures, feature gaps, minor issues</t>
+          <t>"dot_xpu_mkl" kernel NotImplementedError when call</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
@@ -988,12 +993,12 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>Dtype/Precision Issue - "dot_xpu_mkl" not implemented for 'Long' dtype on XPU</t>
+          <t>The error "dot_xpu_mkl not implemented for 'Long'" indicates a missing operator implementation for the Long dtype on XPU. This is a device-specific op dispatch issue, falling under Torch Operations as it relates to operator execution and kernel selection for a specific dtype and device.</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>operator not implemented for Long dtype on XPU</t>
+          <t>Dtype/Precision Issue - The error "dot_xpu_mkl" not implemented for 'Long' indicates a dtype mismatch where the Long tensor is being used with an XPU-specific MKL-optimized dot product operation that does not support integer types. The operation likely expects floating-point dtypes like float32 or b</t>
         </is>
       </c>
     </row>

</xml_diff>